<commit_message>
15.06 update from last week
</commit_message>
<xml_diff>
--- a/appliances_usage.xlsx
+++ b/appliances_usage.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-4488" yWindow="-21108" windowWidth="38400" windowHeight="19392" firstSheet="1" activeTab="1"/>
+    <workbookView xWindow="-4485" yWindow="-21105" windowWidth="38400" windowHeight="19395" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Usage" sheetId="5" state="hidden" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </definedNames>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId5"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2735,7 +2735,7 @@
     <xf numFmtId="9" fontId="25" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2887,6 +2887,7 @@
     </xf>
     <xf numFmtId="0" fontId="33" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" builtinId="8"/>
@@ -34730,7 +34731,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:BJ18" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="92">
     <pivotField showAll="0"/>
@@ -35584,55 +35585,55 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BP53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="4" max="4" width="20.59765625" customWidth="1"/>
-    <col min="5" max="5" width="14.09765625" customWidth="1"/>
-    <col min="7" max="7" width="16.09765625" customWidth="1"/>
-    <col min="8" max="8" width="16.59765625" customWidth="1"/>
-    <col min="10" max="10" width="18.09765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.625" customWidth="1"/>
+    <col min="5" max="5" width="14.125" customWidth="1"/>
+    <col min="7" max="7" width="16.125" customWidth="1"/>
+    <col min="8" max="8" width="16.625" customWidth="1"/>
+    <col min="10" max="10" width="18.125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" hidden="1" customWidth="1"/>
     <col min="12" max="17" width="0" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="16" hidden="1" customWidth="1"/>
     <col min="19" max="22" width="0" hidden="1" customWidth="1"/>
-    <col min="23" max="24" width="12.09765625" hidden="1" customWidth="1"/>
+    <col min="23" max="24" width="12.125" hidden="1" customWidth="1"/>
     <col min="25" max="25" width="0" hidden="1" customWidth="1"/>
     <col min="26" max="26" width="0" style="12" hidden="1" customWidth="1"/>
-    <col min="27" max="27" width="18.59765625" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="14.09765625" style="7" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.59765625" style="7" customWidth="1"/>
-    <col min="30" max="30" width="13.59765625" customWidth="1"/>
-    <col min="31" max="31" width="14.59765625" customWidth="1"/>
-    <col min="32" max="32" width="13.59765625" hidden="1" customWidth="1"/>
-    <col min="33" max="33" width="19.09765625" hidden="1" customWidth="1"/>
-    <col min="34" max="34" width="10.59765625" hidden="1" customWidth="1"/>
-    <col min="35" max="35" width="13.09765625" hidden="1" customWidth="1"/>
-    <col min="36" max="36" width="22.09765625" hidden="1" customWidth="1"/>
-    <col min="37" max="37" width="10.59765625" hidden="1" customWidth="1"/>
-    <col min="38" max="38" width="18.09765625" customWidth="1"/>
-    <col min="39" max="39" width="14.09765625" customWidth="1"/>
-    <col min="40" max="40" width="9.59765625" customWidth="1"/>
-    <col min="41" max="41" width="19.09765625" customWidth="1"/>
-    <col min="42" max="42" width="12.09765625" customWidth="1"/>
+    <col min="27" max="27" width="18.625" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="14.125" style="7" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.625" style="7" customWidth="1"/>
+    <col min="30" max="30" width="13.625" customWidth="1"/>
+    <col min="31" max="31" width="14.625" customWidth="1"/>
+    <col min="32" max="32" width="13.625" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="19.125" hidden="1" customWidth="1"/>
+    <col min="34" max="34" width="10.625" hidden="1" customWidth="1"/>
+    <col min="35" max="35" width="13.125" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="22.125" hidden="1" customWidth="1"/>
+    <col min="37" max="37" width="10.625" hidden="1" customWidth="1"/>
+    <col min="38" max="38" width="18.125" customWidth="1"/>
+    <col min="39" max="39" width="14.125" customWidth="1"/>
+    <col min="40" max="40" width="9.625" customWidth="1"/>
+    <col min="41" max="41" width="19.125" customWidth="1"/>
+    <col min="42" max="42" width="12.125" customWidth="1"/>
     <col min="44" max="45" width="0" hidden="1" customWidth="1"/>
-    <col min="46" max="47" width="13.09765625" hidden="1" customWidth="1"/>
+    <col min="46" max="47" width="13.125" hidden="1" customWidth="1"/>
     <col min="48" max="51" width="0" hidden="1" customWidth="1"/>
-    <col min="52" max="52" width="13.59765625" style="17" hidden="1" customWidth="1"/>
+    <col min="52" max="52" width="13.625" style="17" hidden="1" customWidth="1"/>
     <col min="53" max="53" width="26.5" hidden="1" customWidth="1"/>
-    <col min="54" max="54" width="20.59765625" hidden="1" customWidth="1"/>
+    <col min="54" max="54" width="20.625" hidden="1" customWidth="1"/>
     <col min="55" max="55" width="0" hidden="1" customWidth="1"/>
-    <col min="56" max="56" width="17.59765625" hidden="1" customWidth="1"/>
-    <col min="57" max="57" width="16.09765625" hidden="1" customWidth="1"/>
-    <col min="58" max="58" width="15.09765625" hidden="1" customWidth="1"/>
-    <col min="59" max="59" width="20.59765625" hidden="1" customWidth="1"/>
-    <col min="60" max="60" width="24.59765625" hidden="1" customWidth="1"/>
-    <col min="61" max="61" width="19.59765625" style="30" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="24.09765625" style="30" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="17.625" hidden="1" customWidth="1"/>
+    <col min="57" max="57" width="16.125" hidden="1" customWidth="1"/>
+    <col min="58" max="58" width="15.125" hidden="1" customWidth="1"/>
+    <col min="59" max="59" width="20.625" hidden="1" customWidth="1"/>
+    <col min="60" max="60" width="24.625" hidden="1" customWidth="1"/>
+    <col min="61" max="61" width="19.625" style="30" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="24.125" style="30" bestFit="1" customWidth="1"/>
     <col min="63" max="65" width="11" style="30"/>
-    <col min="67" max="67" width="25.09765625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="25.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" ht="43.2">
+    <row r="1" spans="1:68" ht="45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -43430,7 +43431,7 @@
         <v>6.7567567567567571E-3</v>
       </c>
     </row>
-    <row r="39" spans="1:66" s="41" customFormat="1" ht="16.8">
+    <row r="39" spans="1:66" s="41" customFormat="1" ht="16.5">
       <c r="A39" s="45" t="s">
         <v>68</v>
       </c>
@@ -43635,7 +43636,7 @@
       </c>
       <c r="BN39" s="43"/>
     </row>
-    <row r="40" spans="1:66" s="41" customFormat="1" ht="16.8">
+    <row r="40" spans="1:66" s="41" customFormat="1" ht="16.5">
       <c r="A40" s="45" t="s">
         <v>68</v>
       </c>
@@ -43840,7 +43841,7 @@
       </c>
       <c r="BN40" s="43"/>
     </row>
-    <row r="41" spans="1:66" s="41" customFormat="1" ht="16.8">
+    <row r="41" spans="1:66" s="41" customFormat="1" ht="16.5">
       <c r="A41" s="45" t="s">
         <v>68</v>
       </c>
@@ -44049,7 +44050,7 @@
         <v>2.0421052631578922</v>
       </c>
     </row>
-    <row r="42" spans="1:66" s="41" customFormat="1" ht="16.8">
+    <row r="42" spans="1:66" s="41" customFormat="1" ht="16.5">
       <c r="A42" s="45" t="s">
         <v>68</v>
       </c>
@@ -46535,59 +46536,59 @@
   <dimension ref="A1:CH51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="5" max="5" width="24.59765625" customWidth="1"/>
-    <col min="6" max="6" width="17.59765625" customWidth="1"/>
-    <col min="7" max="7" width="14.09765625" customWidth="1"/>
+    <col min="5" max="5" width="24.625" customWidth="1"/>
+    <col min="6" max="6" width="17.625" customWidth="1"/>
+    <col min="7" max="7" width="14.125" customWidth="1"/>
     <col min="8" max="8" width="16.5" customWidth="1"/>
     <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="16.09765625" customWidth="1"/>
-    <col min="11" max="11" width="15.09765625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.59765625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.09765625" customWidth="1"/>
+    <col min="10" max="10" width="16.125" customWidth="1"/>
+    <col min="11" max="11" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.125" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
-    <col min="16" max="16" width="14.59765625" customWidth="1"/>
-    <col min="17" max="17" width="13.09765625" customWidth="1"/>
+    <col min="16" max="16" width="14.625" customWidth="1"/>
+    <col min="17" max="17" width="13.125" customWidth="1"/>
     <col min="18" max="18" width="15" customWidth="1"/>
-    <col min="19" max="19" width="14.09765625" customWidth="1"/>
+    <col min="19" max="19" width="14.125" customWidth="1"/>
     <col min="20" max="20" width="11" customWidth="1"/>
-    <col min="21" max="21" width="21.09765625" customWidth="1"/>
+    <col min="21" max="21" width="21.125" customWidth="1"/>
     <col min="22" max="22" width="16" customWidth="1"/>
-    <col min="23" max="23" width="14.59765625" customWidth="1"/>
+    <col min="23" max="23" width="14.625" customWidth="1"/>
     <col min="24" max="24" width="12.5" customWidth="1"/>
     <col min="25" max="33" width="11" customWidth="1"/>
     <col min="34" max="35" width="16" customWidth="1"/>
     <col min="36" max="39" width="11" customWidth="1"/>
-    <col min="40" max="41" width="12.09765625" customWidth="1"/>
+    <col min="40" max="41" width="12.125" customWidth="1"/>
     <col min="42" max="42" width="11" customWidth="1"/>
-    <col min="43" max="43" width="27.59765625" customWidth="1"/>
-    <col min="44" max="44" width="41.09765625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="54.59765625" customWidth="1"/>
+    <col min="43" max="43" width="27.625" customWidth="1"/>
+    <col min="44" max="44" width="41.125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="54.625" customWidth="1"/>
     <col min="46" max="46" width="21" customWidth="1"/>
-    <col min="47" max="47" width="26.59765625" style="7" customWidth="1"/>
-    <col min="48" max="48" width="14.09765625" style="7" customWidth="1"/>
-    <col min="49" max="49" width="13.09765625" customWidth="1"/>
-    <col min="50" max="50" width="9.59765625" customWidth="1"/>
+    <col min="47" max="47" width="26.625" style="7" customWidth="1"/>
+    <col min="48" max="48" width="14.125" style="7" customWidth="1"/>
+    <col min="49" max="49" width="13.125" customWidth="1"/>
+    <col min="50" max="50" width="9.625" customWidth="1"/>
     <col min="51" max="51" width="17" customWidth="1"/>
     <col min="52" max="52" width="9"/>
-    <col min="53" max="54" width="14.09765625" customWidth="1"/>
-    <col min="55" max="55" width="13.59765625" customWidth="1"/>
-    <col min="56" max="56" width="12.59765625" customWidth="1"/>
-    <col min="57" max="57" width="10.59765625" customWidth="1"/>
+    <col min="53" max="54" width="14.125" customWidth="1"/>
+    <col min="55" max="55" width="13.625" customWidth="1"/>
+    <col min="56" max="56" width="12.625" customWidth="1"/>
+    <col min="57" max="57" width="10.625" customWidth="1"/>
     <col min="58" max="58" width="13" customWidth="1"/>
-    <col min="59" max="60" width="10.59765625" customWidth="1"/>
-    <col min="61" max="62" width="11.09765625" customWidth="1"/>
+    <col min="59" max="60" width="10.625" customWidth="1"/>
+    <col min="61" max="62" width="11.125" customWidth="1"/>
     <col min="63" max="64" width="11" customWidth="1"/>
-    <col min="65" max="65" width="12.59765625" customWidth="1"/>
-    <col min="66" max="66" width="18.09765625" customWidth="1"/>
-    <col min="67" max="67" width="22.09765625" customWidth="1"/>
-    <col min="68" max="68" width="15.09765625" customWidth="1"/>
+    <col min="65" max="65" width="12.625" customWidth="1"/>
+    <col min="66" max="66" width="18.125" customWidth="1"/>
+    <col min="67" max="67" width="22.125" customWidth="1"/>
+    <col min="68" max="68" width="15.125" customWidth="1"/>
     <col min="69" max="69" width="18" customWidth="1"/>
-    <col min="70" max="70" width="17.09765625" customWidth="1"/>
-    <col min="71" max="71" width="21.09765625" customWidth="1"/>
-    <col min="72" max="72" width="10.09765625" customWidth="1"/>
+    <col min="70" max="70" width="17.125" customWidth="1"/>
+    <col min="71" max="71" width="21.125" customWidth="1"/>
+    <col min="72" max="72" width="10.125" customWidth="1"/>
     <col min="73" max="73" width="13" customWidth="1"/>
     <col min="74" max="74" width="14" customWidth="1"/>
-    <col min="75" max="75" width="13.09765625" customWidth="1"/>
+    <col min="75" max="75" width="13.125" customWidth="1"/>
     <col min="82" max="82" width="24" customWidth="1"/>
   </cols>
   <sheetData>
@@ -46851,7 +46852,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="2" spans="1:86" ht="15.6">
+    <row r="2" spans="1:86">
       <c r="A2" s="11" t="s">
         <v>68</v>
       </c>
@@ -47108,7 +47109,7 @@
         <v>3.8937777431664201E-5</v>
       </c>
     </row>
-    <row r="3" spans="1:86" ht="15.6">
+    <row r="3" spans="1:86">
       <c r="A3" s="11" t="s">
         <v>68</v>
       </c>
@@ -47365,7 +47366,7 @@
         <v>3.8937777431664201E-5</v>
       </c>
     </row>
-    <row r="4" spans="1:86" ht="15.6">
+    <row r="4" spans="1:86">
       <c r="A4" s="11" t="s">
         <v>68</v>
       </c>
@@ -47622,7 +47623,7 @@
         <v>3.8937777431664201E-5</v>
       </c>
     </row>
-    <row r="5" spans="1:86" ht="15.6">
+    <row r="5" spans="1:86">
       <c r="A5" s="11" t="s">
         <v>68</v>
       </c>
@@ -47879,7 +47880,7 @@
         <v>3.8937777431664201E-5</v>
       </c>
     </row>
-    <row r="6" spans="1:86" ht="15.6">
+    <row r="6" spans="1:86">
       <c r="A6" s="11" t="s">
         <v>68</v>
       </c>
@@ -48136,7 +48137,7 @@
         <v>4.0133242364650637E-5</v>
       </c>
     </row>
-    <row r="7" spans="1:86" ht="15.6">
+    <row r="7" spans="1:86">
       <c r="A7" s="11" t="s">
         <v>68</v>
       </c>
@@ -48393,7 +48394,7 @@
         <v>4.4202802457675817E-5</v>
       </c>
     </row>
-    <row r="8" spans="1:86" s="105" customFormat="1" ht="15.6">
+    <row r="8" spans="1:86" s="105" customFormat="1">
       <c r="A8" s="11" t="s">
         <v>68</v>
       </c>
@@ -48653,7 +48654,7 @@
         <v>3.8937777431664201E-5</v>
       </c>
     </row>
-    <row r="9" spans="1:86" s="105" customFormat="1" ht="15.6">
+    <row r="9" spans="1:86" s="105" customFormat="1">
       <c r="A9" s="11" t="s">
         <v>68</v>
       </c>
@@ -48913,7 +48914,7 @@
         <v>3.8937777431664201E-5</v>
       </c>
     </row>
-    <row r="10" spans="1:86" s="105" customFormat="1" ht="15.6">
+    <row r="10" spans="1:86" s="105" customFormat="1">
       <c r="A10" s="11" t="s">
         <v>68</v>
       </c>
@@ -49173,7 +49174,7 @@
         <v>4.0133242364650637E-5</v>
       </c>
     </row>
-    <row r="11" spans="1:86" s="105" customFormat="1" ht="15.6">
+    <row r="11" spans="1:86" s="105" customFormat="1">
       <c r="A11" s="11" t="s">
         <v>68</v>
       </c>
@@ -49433,7 +49434,7 @@
         <v>4.8550759819391176E-5</v>
       </c>
     </row>
-    <row r="12" spans="1:86" ht="15.6">
+    <row r="12" spans="1:86">
       <c r="A12" s="11" t="s">
         <v>68</v>
       </c>
@@ -49690,7 +49691,7 @@
         <v>4.8550759819391176E-5</v>
       </c>
     </row>
-    <row r="13" spans="1:86" s="107" customFormat="1" ht="15.6">
+    <row r="13" spans="1:86" s="107" customFormat="1">
       <c r="A13" s="11" t="s">
         <v>68</v>
       </c>
@@ -49950,7 +49951,7 @@
         <v>4.8550759819391176E-5</v>
       </c>
     </row>
-    <row r="14" spans="1:86" ht="15.6">
+    <row r="14" spans="1:86">
       <c r="A14" t="s">
         <v>68</v>
       </c>
@@ -50205,7 +50206,7 @@
         <v>5.6882821387940839E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:86" ht="15.6">
+    <row r="15" spans="1:86">
       <c r="A15" t="s">
         <v>68</v>
       </c>
@@ -50460,7 +50461,7 @@
         <v>5.6882821387940839E-4</v>
       </c>
     </row>
-    <row r="16" spans="1:86" ht="15.6">
+    <row r="16" spans="1:86">
       <c r="A16" t="s">
         <v>68</v>
       </c>
@@ -50715,7 +50716,7 @@
         <v>1.1061946902654867E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:86" ht="15.6">
+    <row r="17" spans="1:86">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -50970,7 +50971,7 @@
         <v>1.1061946902654867E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:86" s="107" customFormat="1" ht="15.6">
+    <row r="18" spans="1:86" s="107" customFormat="1">
       <c r="A18" s="11" t="s">
         <v>68</v>
       </c>
@@ -51492,7 +51493,7 @@
         <v>2.6660978991148553E-5</v>
       </c>
     </row>
-    <row r="20" spans="1:86" s="107" customFormat="1" ht="15.6">
+    <row r="20" spans="1:86" s="107" customFormat="1">
       <c r="A20" s="11" t="s">
         <v>68</v>
       </c>
@@ -51753,7 +51754,7 @@
         <v>1.4545242978283952E-5</v>
       </c>
     </row>
-    <row r="21" spans="1:86" ht="15.6">
+    <row r="21" spans="1:86">
       <c r="A21" s="11" t="s">
         <v>68</v>
       </c>
@@ -52011,7 +52012,7 @@
         <v>3.0061626333984669E-5</v>
       </c>
     </row>
-    <row r="22" spans="1:86" ht="15.6">
+    <row r="22" spans="1:86">
       <c r="A22" s="11" t="s">
         <v>68</v>
       </c>
@@ -52104,7 +52105,7 @@
         <v>0</v>
       </c>
       <c r="AF22" s="101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG22" s="101" t="s">
         <v>267</v>
@@ -52270,7 +52271,7 @@
         <v>1.953125E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:86" ht="15.6">
+    <row r="23" spans="1:86">
       <c r="A23" s="11" t="s">
         <v>68</v>
       </c>
@@ -52363,7 +52364,7 @@
         <v>0</v>
       </c>
       <c r="AF23" s="101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG23" s="101" t="s">
         <v>267</v>
@@ -52529,7 +52530,7 @@
         <v>1.953125E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:86" ht="15.6">
+    <row r="24" spans="1:86">
       <c r="A24" s="11" t="s">
         <v>68</v>
       </c>
@@ -52549,7 +52550,7 @@
       <c r="G24" t="s">
         <v>271</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24" s="123" t="s">
         <v>272</v>
       </c>
       <c r="I24" s="101">
@@ -52616,13 +52617,13 @@
         <v>0</v>
       </c>
       <c r="AD24" s="101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE24" s="101">
         <v>0</v>
       </c>
       <c r="AF24" s="101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG24" s="101" t="s">
         <v>274</v>
@@ -52873,13 +52874,13 @@
         <v>0</v>
       </c>
       <c r="AD25" s="101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE25" s="101">
         <v>0</v>
       </c>
       <c r="AF25" s="101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG25" s="101" t="s">
         <v>277</v>
@@ -53043,7 +53044,7 @@
         <v>4.1152263374485596E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:86" ht="15.6">
+    <row r="26" spans="1:86">
       <c r="A26" s="11" t="s">
         <v>68</v>
       </c>
@@ -53130,13 +53131,13 @@
         <v>0</v>
       </c>
       <c r="AD26" s="101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE26" s="101">
         <v>0</v>
       </c>
       <c r="AF26" s="101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG26" s="101" t="s">
         <v>277</v>
@@ -53300,7 +53301,7 @@
         <v>4.0950040950040953E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:86" ht="15.6">
+    <row r="27" spans="1:86">
       <c r="A27" s="11" t="s">
         <v>68</v>
       </c>
@@ -53387,13 +53388,13 @@
         <v>0</v>
       </c>
       <c r="AD27" s="101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE27" s="101">
         <v>0</v>
       </c>
       <c r="AF27" s="101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG27" s="101" t="s">
         <v>277</v>
@@ -53557,7 +53558,7 @@
         <v>4.1152263374485596E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:86" ht="15.6">
+    <row r="28" spans="1:86">
       <c r="A28" s="94" t="s">
         <v>68</v>
       </c>
@@ -53817,7 +53818,7 @@
         <v>3.2573289902280132E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:86" ht="15.6">
+    <row r="29" spans="1:86">
       <c r="A29" s="94" t="s">
         <v>68</v>
       </c>
@@ -54077,7 +54078,7 @@
         <v>3.2573289902280132E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:86" ht="15.6">
+    <row r="30" spans="1:86">
       <c r="A30" s="94" t="s">
         <v>68</v>
       </c>
@@ -54337,7 +54338,7 @@
         <v>3.2573289902280132E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:86" ht="15.6">
+    <row r="31" spans="1:86">
       <c r="A31" s="94" t="s">
         <v>68</v>
       </c>
@@ -54596,7 +54597,7 @@
         <v>7.1839080459770114E-5</v>
       </c>
     </row>
-    <row r="32" spans="1:86" ht="15.6">
+    <row r="32" spans="1:86">
       <c r="A32" t="s">
         <v>68</v>
       </c>
@@ -54851,7 +54852,7 @@
         <v>1.0448480111840532E-6</v>
       </c>
     </row>
-    <row r="33" spans="1:86" ht="15.6">
+    <row r="33" spans="1:86">
       <c r="A33" t="s">
         <v>68</v>
       </c>
@@ -55106,7 +55107,7 @@
         <v>1.0448480111840532E-6</v>
       </c>
     </row>
-    <row r="34" spans="1:86" ht="15.6">
+    <row r="34" spans="1:86">
       <c r="A34" t="s">
         <v>68</v>
       </c>
@@ -55361,7 +55362,7 @@
         <v>1.0448480111840532E-6</v>
       </c>
     </row>
-    <row r="35" spans="1:86" ht="15.6">
+    <row r="35" spans="1:86">
       <c r="A35" t="s">
         <v>68</v>
       </c>
@@ -56132,43 +56133,43 @@
         <v>2.5188916876574307E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:86" ht="15.6">
+    <row r="38" spans="1:86">
       <c r="M38" s="18"/>
     </row>
-    <row r="39" spans="1:86" ht="15.6">
+    <row r="39" spans="1:86">
       <c r="M39" s="18"/>
     </row>
-    <row r="40" spans="1:86" ht="15.6">
+    <row r="40" spans="1:86">
       <c r="M40" s="18"/>
     </row>
-    <row r="41" spans="1:86" ht="15.6">
+    <row r="41" spans="1:86">
       <c r="M41" s="18"/>
     </row>
-    <row r="42" spans="1:86" ht="15.6">
+    <row r="42" spans="1:86">
       <c r="M42" s="18"/>
     </row>
-    <row r="43" spans="1:86" ht="15.6">
+    <row r="43" spans="1:86">
       <c r="M43" s="18"/>
     </row>
-    <row r="44" spans="1:86" ht="15.6">
+    <row r="44" spans="1:86">
       <c r="M44" s="18"/>
     </row>
-    <row r="45" spans="1:86" ht="15.6">
+    <row r="45" spans="1:86">
       <c r="M45" s="18"/>
     </row>
-    <row r="46" spans="1:86" ht="15.6">
+    <row r="46" spans="1:86">
       <c r="M46" s="18"/>
     </row>
     <row r="47" spans="1:86" ht="15.75" customHeight="1">
       <c r="M47" s="18"/>
       <c r="BX47" s="30"/>
     </row>
-    <row r="48" spans="1:86" ht="15.6">
+    <row r="48" spans="1:86">
       <c r="M48" s="18"/>
       <c r="BA48" s="117"/>
       <c r="BB48" s="117"/>
     </row>
-    <row r="49" spans="13:54" ht="15.6">
+    <row r="49" spans="13:54">
       <c r="M49" s="18"/>
       <c r="BA49" s="117"/>
       <c r="BB49" s="117"/>
@@ -56176,7 +56177,7 @@
     <row r="50" spans="13:54" ht="15.75" customHeight="1">
       <c r="M50" s="18"/>
     </row>
-    <row r="51" spans="13:54" ht="15.6">
+    <row r="51" spans="13:54">
       <c r="M51" s="18"/>
       <c r="BA51" s="118"/>
       <c r="BB51" s="118"/>
@@ -56350,70 +56351,70 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BJ18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="28.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.09765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.59765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.3984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.8984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="30" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="26.59765625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.3984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.09765625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.59765625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="28.09765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.09765625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="26.625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="28.125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="15" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.375" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.8984375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.8984375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="11" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="23.8984375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.8984375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="22.59765625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="15.8984375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="17.09765625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="23.875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="17.125" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="17" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="13.59765625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="18.8984375" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="9.3984375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="9.09765625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="36.3984375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="18.875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="9.125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="36.375" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="29" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="17.8984375" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="21.8984375" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="20.09765625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="21.875" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="20.125" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="15" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13.3984375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="21.8984375" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="21.875" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="36.5" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="23.8984375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="17.09765625" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="29.59765625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="23.875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="29.625" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="33" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="35.5" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="21.8984375" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="24.3984375" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="17.8984375" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="25.8984375" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="21.875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="24.375" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="25.875" bestFit="1" customWidth="1"/>
     <col min="58" max="58" width="35" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="26.3984375" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.3984375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="26.375" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.375" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="15.625" bestFit="1" customWidth="1"/>
     <col min="63" max="64" width="18.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -59255,15 +59256,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S99"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="3" max="3" width="15.5" customWidth="1"/>
-    <col min="5" max="5" width="19.59765625" customWidth="1"/>
+    <col min="5" max="5" width="19.625" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="18.09765625" style="26" customWidth="1"/>
+    <col min="7" max="7" width="18.125" style="26" customWidth="1"/>
     <col min="8" max="8" width="20.5" customWidth="1"/>
-    <col min="9" max="9" width="14.09765625" customWidth="1"/>
-    <col min="10" max="10" width="15.09765625" customWidth="1"/>
+    <col min="9" max="9" width="14.125" customWidth="1"/>
+    <col min="10" max="10" width="15.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -59322,7 +59323,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="31.2">
+    <row r="2" spans="1:19" ht="31.5">
       <c r="A2">
         <v>0</v>
       </c>
@@ -59378,7 +59379,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="31.2">
+    <row r="3" spans="1:19" ht="31.5">
       <c r="A3">
         <v>1</v>
       </c>
@@ -59434,7 +59435,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="46.8">
+    <row r="4" spans="1:19" ht="47.25">
       <c r="A4" t="s">
         <v>73</v>
       </c>
@@ -59484,7 +59485,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="46.8">
+    <row r="5" spans="1:19" ht="47.25">
       <c r="D5" t="s">
         <v>293</v>
       </c>

</xml_diff>